<commit_message>
Actualizar excel Capas SIG
agregar columna con link a github
</commit_message>
<xml_diff>
--- a/Capas_SIG.xlsx
+++ b/Capas_SIG.xlsx
@@ -1,23 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fer\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7769FEEC-C6A1-44A9-A311-940506A5E244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="125725"/>
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1872" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1874" uniqueCount="605">
   <si>
     <t>orden original</t>
   </si>
@@ -1834,13 +1828,19 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>Link GitHub</t>
+  </si>
+  <si>
+    <t>Capa_nombre</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1854,6 +1854,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1885,10 +1892,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1899,30 +1910,19 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="4">
     <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="255" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1944,19 +1944,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1971,24 +1958,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:O191" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:O191" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="orden original"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Clase"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Subclase"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Geometría"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Nombre de la capa base"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Acronimo"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Config Manual"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Config Minima"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Config Estandar"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="50k"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="100k"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="250k"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="500k"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Button CSV completo"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Link CSV"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:Q191" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:Q191">
+    <filterColumn colId="15"/>
+    <filterColumn colId="16"/>
+  </autoFilter>
+  <tableColumns count="17">
+    <tableColumn id="1" name="orden original"/>
+    <tableColumn id="2" name="Clase"/>
+    <tableColumn id="3" name="Subclase"/>
+    <tableColumn id="4" name="Geometría"/>
+    <tableColumn id="5" name="Nombre de la capa base"/>
+    <tableColumn id="6" name="Acronimo"/>
+    <tableColumn id="7" name="Config Manual"/>
+    <tableColumn id="8" name="Config Minima"/>
+    <tableColumn id="9" name="Config Estandar"/>
+    <tableColumn id="10" name="50k"/>
+    <tableColumn id="11" name="100k"/>
+    <tableColumn id="12" name="250k"/>
+    <tableColumn id="13" name="500k"/>
+    <tableColumn id="14" name="Button CSV completo"/>
+    <tableColumn id="15" name="Link CSV"/>
+    <tableColumn id="16" name="Capa_nombre"/>
+    <tableColumn id="17" name="Link GitHub" dataDxfId="0">
+      <calculatedColumnFormula>"https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/" &amp; P2 &amp; ".zip"</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2037,7 +2031,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -2089,7 +2083,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -2303,30 +2297,32 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O191"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q191"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" customWidth="1"/>
-    <col min="2" max="2" width="22.21875" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="1" max="1" width="13.75" customWidth="1"/>
+    <col min="2" max="2" width="22.25" customWidth="1"/>
+    <col min="3" max="3" width="23.875" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.6640625" customWidth="1"/>
-    <col min="8" max="8" width="18.21875" customWidth="1"/>
-    <col min="9" max="9" width="19.77734375" customWidth="1"/>
-    <col min="14" max="14" width="19.6640625" customWidth="1"/>
+    <col min="6" max="6" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.625" customWidth="1"/>
+    <col min="8" max="8" width="18.25" customWidth="1"/>
+    <col min="9" max="9" width="19.75" customWidth="1"/>
+    <col min="14" max="14" width="19.625" customWidth="1"/>
+    <col min="16" max="16" width="31.875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="111.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2372,8 +2368,14 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P1" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2">
         <v>69</v>
       </c>
@@ -2407,11 +2409,19 @@
       <c r="N2" t="s">
         <v>20</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P2" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_actividad_agropecuaria_AL270</v>
+      </c>
+      <c r="Q2" s="5" t="str">
+        <f t="shared" ref="Q2:Q65" si="0">"https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/" &amp; P2 &amp; ".zip"</f>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_actividad_agropecuaria_AL270.zip</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3">
         <v>93</v>
       </c>
@@ -2448,8 +2458,16 @@
       <c r="O3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P3" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_actividad_agropecuaria_AJ110</v>
+      </c>
+      <c r="Q3" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_actividad_agropecuaria_AJ110.zip</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4">
         <v>94</v>
       </c>
@@ -2486,8 +2504,16 @@
       <c r="O4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P4" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_actividad_agropecuaria_AJ110</v>
+      </c>
+      <c r="Q4" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_actividad_agropecuaria_AJ110.zip</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5">
         <v>111</v>
       </c>
@@ -2524,8 +2550,16 @@
       <c r="O5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P5" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_actividad_agropecuaria_AJ050</v>
+      </c>
+      <c r="Q5" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_actividad_agropecuaria_AJ050.zip</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6">
         <v>6</v>
       </c>
@@ -2562,8 +2596,16 @@
       <c r="O6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P6" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_transporte_aereo_GB001</v>
+      </c>
+      <c r="Q6" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_transporte_aereo_GB001.zip</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7">
         <v>7</v>
       </c>
@@ -2600,8 +2642,16 @@
       <c r="O7" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P7" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_transporte_aereo_GB005</v>
+      </c>
+      <c r="Q7" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_transporte_aereo_GB005.zip</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8">
         <v>86</v>
       </c>
@@ -2638,8 +2688,16 @@
       <c r="O8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P8" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_transporte_aereo_GB035</v>
+      </c>
+      <c r="Q8" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_transporte_aereo_GB035.zip</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9">
         <v>122</v>
       </c>
@@ -2676,8 +2734,16 @@
       <c r="O9" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P9" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_transporte_aereo_GB055</v>
+      </c>
+      <c r="Q9" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_transporte_aereo_GB055.zip</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10">
         <v>4</v>
       </c>
@@ -2714,8 +2780,16 @@
       <c r="O10" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P10" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_aguas_continentales_BH030</v>
+      </c>
+      <c r="Q10" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_aguas_continentales_BH030.zip</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11">
         <v>5</v>
       </c>
@@ -2752,8 +2826,16 @@
       <c r="O11" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P11" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_aguas_continentales_BH010</v>
+      </c>
+      <c r="Q11" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_aguas_continentales_BH010.zip</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12">
         <v>25</v>
       </c>
@@ -2787,8 +2869,16 @@
       <c r="O12" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P12" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_aguas_continentales_BH020</v>
+      </c>
+      <c r="Q12" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_aguas_continentales_BH020.zip</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13">
         <v>26</v>
       </c>
@@ -2822,8 +2912,16 @@
       <c r="O13" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P13" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_aguas_continentales_BH020</v>
+      </c>
+      <c r="Q13" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_aguas_continentales_BH020.zip</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14">
         <v>32</v>
       </c>
@@ -2857,8 +2955,16 @@
       <c r="O14" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P14" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_aguas_continentales_BH180</v>
+      </c>
+      <c r="Q14" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_aguas_continentales_BH180.zip</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15">
         <v>43</v>
       </c>
@@ -2892,8 +2998,16 @@
       <c r="O15" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P15" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_aguas_continentales_BH140</v>
+      </c>
+      <c r="Q15" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_aguas_continentales_BH140.zip</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16">
         <v>44</v>
       </c>
@@ -2927,8 +3041,16 @@
       <c r="O16" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P16" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_aguas_continentales_BH140</v>
+      </c>
+      <c r="Q16" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_aguas_continentales_BH140.zip</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17">
         <v>45</v>
       </c>
@@ -2962,8 +3084,16 @@
       <c r="O17" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P17" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_aguas_continentales_perenne</v>
+      </c>
+      <c r="Q17" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_aguas_continentales_perenne.zip</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18">
         <v>53</v>
       </c>
@@ -2997,8 +3127,16 @@
       <c r="O18" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P18" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_aguas_continentales_BH051</v>
+      </c>
+      <c r="Q18" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_aguas_continentales_BH051.zip</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19">
         <v>63</v>
       </c>
@@ -3032,8 +3170,16 @@
       <c r="O19" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P19" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_aguas_continentales_BH130</v>
+      </c>
+      <c r="Q19" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_aguas_continentales_BH130.zip</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20">
         <v>64</v>
       </c>
@@ -3067,8 +3213,16 @@
       <c r="O20" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P20" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_aguas_continentales_BH130</v>
+      </c>
+      <c r="Q20" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_aguas_continentales_BH130.zip</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21">
         <v>65</v>
       </c>
@@ -3102,8 +3256,16 @@
       <c r="O21" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P21" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_aguas_continentales_041101</v>
+      </c>
+      <c r="Q21" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_aguas_continentales_041101.zip</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22">
         <v>67</v>
       </c>
@@ -3137,8 +3299,16 @@
       <c r="O22" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P22" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_aguas_continentales_041101</v>
+      </c>
+      <c r="Q22" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_aguas_continentales_041101.zip</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23">
         <v>68</v>
       </c>
@@ -3172,8 +3342,16 @@
       <c r="O23" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P23" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_aguas_continentales_perenne</v>
+      </c>
+      <c r="Q23" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_aguas_continentales_perenne.zip</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24">
         <v>81</v>
       </c>
@@ -3207,8 +3385,16 @@
       <c r="O24" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P24" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_aguas_continentales_BH170</v>
+      </c>
+      <c r="Q24" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_aguas_continentales_BH170.zip</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25">
         <v>116</v>
       </c>
@@ -3242,8 +3428,16 @@
       <c r="O25" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P25" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_aguas_continentales_BH170</v>
+      </c>
+      <c r="Q25" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_aguas_continentales_BH170.zip</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26">
         <v>175</v>
       </c>
@@ -3277,8 +3471,16 @@
       <c r="O26" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P26" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_almacenamiento_y_logistica_AM080</v>
+      </c>
+      <c r="Q26" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_almacenamiento_y_logistica_AM080.zip</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27">
         <v>176</v>
       </c>
@@ -3312,8 +3514,16 @@
       <c r="O27" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P27" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_almacenamiento_y_logistica_AM070</v>
+      </c>
+      <c r="Q27" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_almacenamiento_y_logistica_AM070.zip</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28">
         <v>40</v>
       </c>
@@ -3347,8 +3557,16 @@
       <c r="O28" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P28" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>complejos_fronterizos</v>
+      </c>
+      <c r="Q28" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/complejos_fronterizos.zip</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29">
         <v>20</v>
       </c>
@@ -3382,8 +3600,16 @@
       <c r="O29" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P29" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>bahra_base_antartica</v>
+      </c>
+      <c r="Q29" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/bahra_base_antartica.zip</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30">
         <v>56</v>
       </c>
@@ -3417,8 +3643,16 @@
       <c r="O30" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P30" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_asentamientos_y_edificios_AL015</v>
+      </c>
+      <c r="Q30" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_asentamientos_y_edificios_AL015.zip</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31">
         <v>57</v>
       </c>
@@ -3452,8 +3686,16 @@
       <c r="O31" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P31" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_asentamientos_y_edificios_020102</v>
+      </c>
+      <c r="Q31" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_asentamientos_y_edificios_020102.zip</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32">
         <v>61</v>
       </c>
@@ -3487,8 +3729,16 @@
       <c r="O32" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P32" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_asentamientos_y_edificios_020101</v>
+      </c>
+      <c r="Q32" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_asentamientos_y_edificios_020101.zip</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33">
         <v>103</v>
       </c>
@@ -3522,8 +3772,16 @@
       <c r="O33" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P33" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>localidad_bahra</v>
+      </c>
+      <c r="Q33" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/localidad_bahra.zip</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34">
         <v>119</v>
       </c>
@@ -3557,8 +3815,16 @@
       <c r="O34" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P34" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>bahra_paraje</v>
+      </c>
+      <c r="Q34" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/bahra_paraje.zip</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35">
         <v>131</v>
       </c>
@@ -3592,8 +3858,16 @@
       <c r="O35" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P35" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_asentamientos_y_edificios_020105</v>
+      </c>
+      <c r="Q35" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_asentamientos_y_edificios_020105.zip</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36">
         <v>168</v>
       </c>
@@ -3627,8 +3901,16 @@
       <c r="O36" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P36" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_asentamientos_y_edificios_ruina</v>
+      </c>
+      <c r="Q36" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_asentamientos_y_edificios_ruina.zip</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37">
         <v>173</v>
       </c>
@@ -3662,8 +3944,16 @@
       <c r="O37" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P37" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_asentamientos_y_edificios_ruina</v>
+      </c>
+      <c r="Q37" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_asentamientos_y_edificios_ruina.zip</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38">
         <v>174</v>
       </c>
@@ -3697,8 +3987,16 @@
       <c r="O38" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P38" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>sublocalidad_entidad_bahra</v>
+      </c>
+      <c r="Q38" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/sublocalidad_entidad_bahra.zip</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39">
         <v>177</v>
       </c>
@@ -3732,8 +4030,16 @@
       <c r="O39" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P39" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_asentamientos_y_edificios_020108</v>
+      </c>
+      <c r="Q39" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_asentamientos_y_edificios_020108.zip</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40">
         <v>16</v>
       </c>
@@ -3767,8 +4073,16 @@
       <c r="O40" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P40" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>ayuda_a_la_navegacion_BC101</v>
+      </c>
+      <c r="Q40" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/ayuda_a_la_navegacion_BC101.zip</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17">
       <c r="A41">
         <v>23</v>
       </c>
@@ -3802,8 +4116,16 @@
       <c r="O41" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P41" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>ayuda_a_la_navegacion_BC020</v>
+      </c>
+      <c r="Q41" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/ayuda_a_la_navegacion_BC020.zip</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17">
       <c r="A42">
         <v>78</v>
       </c>
@@ -3837,8 +4159,16 @@
       <c r="O42" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P42" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>ayuda_a_la_navegacion_BC050</v>
+      </c>
+      <c r="Q42" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/ayuda_a_la_navegacion_BC050.zip</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43">
         <v>36</v>
       </c>
@@ -3872,8 +4202,16 @@
       <c r="O43" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P43" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_ciencia_y_educacion_AL295</v>
+      </c>
+      <c r="Q43" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_ciencia_y_educacion_AL295.zip</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17">
       <c r="A44">
         <v>70</v>
       </c>
@@ -3907,8 +4245,16 @@
       <c r="O44" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P44" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_ciencia_y_educacion_AL295</v>
+      </c>
+      <c r="Q44" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_ciencia_y_educacion_AL295.zip</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17">
       <c r="A45">
         <v>182</v>
       </c>
@@ -3942,8 +4288,16 @@
       <c r="O45" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P45" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_ciencia_y_educacion_020602</v>
+      </c>
+      <c r="Q45" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_ciencia_y_educacion_020602.zip</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46">
         <v>10</v>
       </c>
@@ -3977,8 +4331,16 @@
       <c r="O46" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P46" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_comunicacion_AT010</v>
+      </c>
+      <c r="Q46" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_comunicacion_AT010.zip</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47">
         <v>179</v>
       </c>
@@ -4012,8 +4374,16 @@
       <c r="O47" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P47" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_comunicacion_AT080</v>
+      </c>
+      <c r="Q47" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_comunicacion_AT080.zip</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48">
         <v>142</v>
       </c>
@@ -4047,8 +4417,16 @@
       <c r="O48" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P48" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>controles_AH070</v>
+      </c>
+      <c r="Q48" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/controles_AH070.zip</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17">
       <c r="A49">
         <v>9</v>
       </c>
@@ -4082,8 +4460,16 @@
       <c r="O49" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P49" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>controles_AH070</v>
+      </c>
+      <c r="Q49" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/controles_AH070.zip</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17">
       <c r="A50">
         <v>139</v>
       </c>
@@ -4114,8 +4500,16 @@
       <c r="O50" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P50" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_cruces_y_enlaces_AQ040</v>
+      </c>
+      <c r="Q50" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_cruces_y_enlaces_AQ040.zip</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17">
       <c r="A51">
         <v>140</v>
       </c>
@@ -4149,8 +4543,16 @@
       <c r="O51" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P51" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_cruces_y_enlaces_AQ040</v>
+      </c>
+      <c r="Q51" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_cruces_y_enlaces_AQ040.zip</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17">
       <c r="A52">
         <v>181</v>
       </c>
@@ -4184,8 +4586,16 @@
       <c r="O52" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P52" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_cruces_y_enlaces_AQ130</v>
+      </c>
+      <c r="Q52" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_cruces_y_enlaces_AQ130.zip</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17">
       <c r="A53">
         <v>183</v>
       </c>
@@ -4219,8 +4629,16 @@
       <c r="O53" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P53" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_cruces_y_enlaces_BH070</v>
+      </c>
+      <c r="Q53" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_cruces_y_enlaces_BH070.zip</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17">
       <c r="A54">
         <v>132</v>
       </c>
@@ -4242,8 +4660,16 @@
       <c r="O54" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P54" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>plantacion_permanente_KB025</v>
+      </c>
+      <c r="Q54" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/plantacion_permanente_KB025.zip</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17">
       <c r="A55">
         <v>178</v>
       </c>
@@ -4265,8 +4691,16 @@
       <c r="O55" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P55" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>terreno_para_cultivo_EA010</v>
+      </c>
+      <c r="Q55" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/terreno_para_cultivo_EA010.zip</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56">
         <v>58</v>
       </c>
@@ -4300,8 +4734,16 @@
       <c r="O56" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P56" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>cultura_y_religion_AL021</v>
+      </c>
+      <c r="Q56" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/cultura_y_religion_AL021.zip</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17">
       <c r="A57">
         <v>62</v>
       </c>
@@ -4335,8 +4777,16 @@
       <c r="O57" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P57" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>cultura_y_religion_AL330</v>
+      </c>
+      <c r="Q57" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/cultura_y_religion_AL330.zip</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17">
       <c r="A58">
         <v>8</v>
       </c>
@@ -4370,8 +4820,16 @@
       <c r="O58" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P58" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>edafologia_afloramiento_rocoso</v>
+      </c>
+      <c r="Q58" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/edafologia_afloramiento_rocoso.zip</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17">
       <c r="A59">
         <v>15</v>
       </c>
@@ -4405,8 +4863,16 @@
       <c r="O59" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P59" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>edafologia_arenal</v>
+      </c>
+      <c r="Q59" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/edafologia_arenal.zip</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17">
       <c r="A60">
         <v>19</v>
       </c>
@@ -4440,8 +4906,16 @@
       <c r="O60" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P60" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>edafologia_barrial_barrizal</v>
+      </c>
+      <c r="Q60" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/edafologia_barrial_barrizal.zip</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17">
       <c r="A61">
         <v>49</v>
       </c>
@@ -4475,8 +4949,16 @@
       <c r="O61" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P61" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>edafologia_cumbre_rocosa</v>
+      </c>
+      <c r="Q61" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/edafologia_cumbre_rocosa.zip</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17">
       <c r="A62">
         <v>121</v>
       </c>
@@ -4510,8 +4992,16 @@
       <c r="O62" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P62" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>edafologia_pedregal</v>
+      </c>
+      <c r="Q62" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/edafologia_pedregal.zip</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17">
       <c r="A63">
         <v>169</v>
       </c>
@@ -4545,8 +5035,16 @@
       <c r="O63" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P63" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>edafologia_salina</v>
+      </c>
+      <c r="Q63" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/edafologia_salina.zip</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17">
       <c r="A64">
         <v>170</v>
       </c>
@@ -4580,8 +5078,16 @@
       <c r="O64" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P64" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>edafologia_salina</v>
+      </c>
+      <c r="Q64" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/edafologia_salina.zip</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17">
       <c r="A65">
         <v>28</v>
       </c>
@@ -4603,8 +5109,16 @@
       <c r="O65" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P65" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>cartas_100000</v>
+      </c>
+      <c r="Q65" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/cartas_100000.zip</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17">
       <c r="A66">
         <v>29</v>
       </c>
@@ -4626,8 +5140,16 @@
       <c r="O66" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P66" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>cartas_250000</v>
+      </c>
+      <c r="Q66" s="5" t="str">
+        <f t="shared" ref="Q66:Q129" si="1">"https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/" &amp; P66 &amp; ".zip"</f>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/cartas_250000.zip</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17">
       <c r="A67">
         <v>30</v>
       </c>
@@ -4649,8 +5171,16 @@
       <c r="O67" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P67" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>cartas_50000</v>
+      </c>
+      <c r="Q67" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/cartas_50000.zip</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17">
       <c r="A68">
         <v>31</v>
       </c>
@@ -4672,8 +5202,16 @@
       <c r="O68" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P68" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>cartas_500000</v>
+      </c>
+      <c r="Q68" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/cartas_500000.zip</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17">
       <c r="A69">
         <v>35</v>
       </c>
@@ -4707,8 +5245,16 @@
       <c r="O69" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P69" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_energia_AD010</v>
+      </c>
+      <c r="Q69" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_energia_AD010.zip</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17">
       <c r="A70">
         <v>102</v>
       </c>
@@ -4742,8 +5288,16 @@
       <c r="O70" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P70" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_energia_AT030</v>
+      </c>
+      <c r="Q70" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_energia_AT030.zip</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17">
       <c r="A71">
         <v>130</v>
       </c>
@@ -4777,8 +5331,16 @@
       <c r="O71" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P71" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_energia_AD030</v>
+      </c>
+      <c r="Q71" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_energia_AD030.zip</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17">
       <c r="A72">
         <v>33</v>
       </c>
@@ -4812,8 +5374,16 @@
       <c r="O72" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P72" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>cultura_y_religion_AL330</v>
+      </c>
+      <c r="Q72" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/cultura_y_religion_AL330.zip</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17">
       <c r="A73">
         <v>34</v>
       </c>
@@ -4847,8 +5417,16 @@
       <c r="O73" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P73" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_equipamiento_AL030</v>
+      </c>
+      <c r="Q73" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_equipamiento_AL030.zip</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17">
       <c r="A74">
         <v>66</v>
       </c>
@@ -4882,8 +5460,16 @@
       <c r="O74" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P74" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_equipamiento_AL170</v>
+      </c>
+      <c r="Q74" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_equipamiento_AL170.zip</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17">
       <c r="A75">
         <v>113</v>
       </c>
@@ -4917,8 +5503,16 @@
       <c r="O75" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P75" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_equipamiento_AL170</v>
+      </c>
+      <c r="Q75" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_equipamiento_AL170.zip</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17">
       <c r="A76">
         <v>163</v>
       </c>
@@ -4952,8 +5546,16 @@
       <c r="O76" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P76" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_equipamiento_AH030</v>
+      </c>
+      <c r="Q76" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_equipamiento_AH030.zip</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17">
       <c r="A77">
         <v>24</v>
       </c>
@@ -4987,8 +5589,16 @@
       <c r="O77" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P77" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_estructura_asociada_AA051</v>
+      </c>
+      <c r="Q77" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_estructura_asociada_AA051.zip</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17">
       <c r="A78">
         <v>54</v>
       </c>
@@ -5022,8 +5632,16 @@
       <c r="O78" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P78" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_estructura_asociada_ducto_subterraneo</v>
+      </c>
+      <c r="Q78" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_estructura_asociada_ducto_subterraneo.zip</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17">
       <c r="A79">
         <v>82</v>
       </c>
@@ -5057,8 +5675,16 @@
       <c r="O79" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P79" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_estructura_asociada_AJ080</v>
+      </c>
+      <c r="Q79" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_estructura_asociada_AJ080.zip</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17">
       <c r="A80">
         <v>123</v>
       </c>
@@ -5092,8 +5718,16 @@
       <c r="O80" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P80" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_estructura_asociada_AQ116</v>
+      </c>
+      <c r="Q80" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_estructura_asociada_AQ116.zip</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17">
       <c r="A81">
         <v>188</v>
       </c>
@@ -5127,8 +5761,16 @@
       <c r="O81" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P81" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_estructura_asociada_010601</v>
+      </c>
+      <c r="Q81" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_estructura_asociada_010601.zip</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17">
       <c r="A82">
         <v>46</v>
       </c>
@@ -5162,8 +5804,16 @@
       <c r="O82" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P82" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>estructuras_operativas_y_defensivas_090102</v>
+      </c>
+      <c r="Q82" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/estructuras_operativas_y_defensivas_090102.zip</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17">
       <c r="A83">
         <v>60</v>
       </c>
@@ -5197,8 +5847,16 @@
       <c r="O83" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P83" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>estructuras_operativas_y_defensivas_090102</v>
+      </c>
+      <c r="Q83" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/estructuras_operativas_y_defensivas_090102.zip</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17">
       <c r="A84">
         <v>92</v>
       </c>
@@ -5232,8 +5890,16 @@
       <c r="O84" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P84" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>estructuras_operativas_y_defensivas_090102</v>
+      </c>
+      <c r="Q84" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/estructuras_operativas_y_defensivas_090102.zip</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17">
       <c r="A85">
         <v>27</v>
       </c>
@@ -5267,8 +5933,16 @@
       <c r="O85" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P85" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_extraccion_AA012</v>
+      </c>
+      <c r="Q85" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_extraccion_AA012.zip</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17">
       <c r="A86">
         <v>109</v>
       </c>
@@ -5302,8 +5976,16 @@
       <c r="O86" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P86" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_extraccion_AA010</v>
+      </c>
+      <c r="Q86" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_extraccion_AA010.zip</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17">
       <c r="A87">
         <v>137</v>
       </c>
@@ -5337,8 +6019,16 @@
       <c r="O87" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P87" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_extraccion_AA050</v>
+      </c>
+      <c r="Q87" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_extraccion_AA050.zip</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17">
       <c r="A88">
         <v>186</v>
       </c>
@@ -5372,8 +6062,16 @@
       <c r="O88" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P88" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_extraccion_AA052</v>
+      </c>
+      <c r="Q88" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_extraccion_AA052.zip</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17">
       <c r="A89">
         <v>12</v>
       </c>
@@ -5407,8 +6105,16 @@
       <c r="O89" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P89" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_fabricacion_y_procesamiento_AC070</v>
+      </c>
+      <c r="Q89" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_fabricacion_y_procesamiento_AC070.zip</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17">
       <c r="A90">
         <v>77</v>
       </c>
@@ -5442,8 +6148,16 @@
       <c r="O90" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P90" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_fabricacion_y_procesamiento_AC000</v>
+      </c>
+      <c r="Q90" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_fabricacion_y_procesamiento_AC000.zip</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17">
       <c r="A91">
         <v>124</v>
       </c>
@@ -5477,8 +6191,16 @@
       <c r="O91" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P91" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_fabricacion_y_procesamiento_AC507</v>
+      </c>
+      <c r="Q91" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_fabricacion_y_procesamiento_AC507.zip</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17">
       <c r="A92">
         <v>125</v>
       </c>
@@ -5512,8 +6234,16 @@
       <c r="O92" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P92" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_fabricacion_y_procesamiento_AC507</v>
+      </c>
+      <c r="Q92" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_fabricacion_y_procesamiento_AC507.zip</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17">
       <c r="A93">
         <v>128</v>
       </c>
@@ -5547,8 +6277,16 @@
       <c r="O93" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P93" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_fabricacion_y_procesamiento_BH220</v>
+      </c>
+      <c r="Q93" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_fabricacion_y_procesamiento_BH220.zip</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17">
       <c r="A94">
         <v>129</v>
       </c>
@@ -5582,8 +6320,16 @@
       <c r="O94" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P94" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_fabricacion_y_procesamiento_BH220</v>
+      </c>
+      <c r="Q94" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_fabricacion_y_procesamiento_BH220.zip</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17">
       <c r="A95">
         <v>71</v>
       </c>
@@ -5617,8 +6363,16 @@
       <c r="O95" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P95" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_transporte_ferroviario_AN070</v>
+      </c>
+      <c r="Q95" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_transporte_ferroviario_AN070.zip</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17">
       <c r="A96">
         <v>79</v>
       </c>
@@ -5652,8 +6406,16 @@
       <c r="O96" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P96" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_transporte_ferroviario_AN010</v>
+      </c>
+      <c r="Q96" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_transporte_ferroviario_AN010.zip</v>
+      </c>
+    </row>
+    <row r="97" spans="1:17">
       <c r="A97">
         <v>2</v>
       </c>
@@ -5687,8 +6449,16 @@
       <c r="O97" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P97" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_geomorfologia_DB120</v>
+      </c>
+      <c r="Q97" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_geomorfologia_DB120.zip</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17">
       <c r="A98">
         <v>13</v>
       </c>
@@ -5722,8 +6492,16 @@
       <c r="O98" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P98" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>area_de_montana</v>
+      </c>
+      <c r="Q98" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/area_de_montana.zip</v>
+      </c>
+    </row>
+    <row r="99" spans="1:17">
       <c r="A99">
         <v>17</v>
       </c>
@@ -5757,8 +6535,16 @@
       <c r="O99" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P99" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_barranca</v>
+      </c>
+      <c r="Q99" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_barranca.zip</v>
+      </c>
+    </row>
+    <row r="100" spans="1:17">
       <c r="A100">
         <v>38</v>
       </c>
@@ -5792,8 +6578,16 @@
       <c r="O100" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P100" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_geomorfologia_NA100</v>
+      </c>
+      <c r="Q100" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_geomorfologia_NA100.zip</v>
+      </c>
+    </row>
+    <row r="101" spans="1:17">
       <c r="A101">
         <v>41</v>
       </c>
@@ -5827,8 +6621,16 @@
       <c r="O101" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P101" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_geomorfologia_NA100</v>
+      </c>
+      <c r="Q101" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_geomorfologia_NA100.zip</v>
+      </c>
+    </row>
+    <row r="102" spans="1:17">
       <c r="A102">
         <v>42</v>
       </c>
@@ -5862,8 +6664,16 @@
       <c r="O102" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P102" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_050206</v>
+      </c>
+      <c r="Q102" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_050206.zip</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17">
       <c r="A103">
         <v>47</v>
       </c>
@@ -5897,8 +6707,16 @@
       <c r="O103" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P103" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_050207</v>
+      </c>
+      <c r="Q103" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_050207.zip</v>
+      </c>
+    </row>
+    <row r="104" spans="1:17">
       <c r="A104">
         <v>48</v>
       </c>
@@ -5932,8 +6750,16 @@
       <c r="O104" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P104" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_050208</v>
+      </c>
+      <c r="Q104" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_050208.zip</v>
+      </c>
+    </row>
+    <row r="105" spans="1:17">
       <c r="A105">
         <v>50</v>
       </c>
@@ -5967,8 +6793,16 @@
       <c r="O105" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P105" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_CA010</v>
+      </c>
+      <c r="Q105" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_CA010.zip</v>
+      </c>
+    </row>
+    <row r="106" spans="1:17">
       <c r="A106">
         <v>80</v>
       </c>
@@ -6002,8 +6836,16 @@
       <c r="O106" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P106" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_CA020</v>
+      </c>
+      <c r="Q106" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_CA020.zip</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17">
       <c r="A107">
         <v>104</v>
       </c>
@@ -6037,8 +6879,16 @@
       <c r="O107" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P107" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_DB001</v>
+      </c>
+      <c r="Q107" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_DB001.zip</v>
+      </c>
+    </row>
+    <row r="108" spans="1:17">
       <c r="A108">
         <v>107</v>
       </c>
@@ -6072,8 +6922,16 @@
       <c r="O108" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P108" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_geomorfologia_DB560</v>
+      </c>
+      <c r="Q108" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_geomorfologia_DB560.zip</v>
+      </c>
+    </row>
+    <row r="109" spans="1:17">
       <c r="A109">
         <v>108</v>
       </c>
@@ -6107,8 +6965,16 @@
       <c r="O109" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P109" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_geomorfologia_DB560</v>
+      </c>
+      <c r="Q109" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_geomorfologia_DB560.zip</v>
+      </c>
+    </row>
+    <row r="110" spans="1:17">
       <c r="A110">
         <v>110</v>
       </c>
@@ -6142,8 +7008,16 @@
       <c r="O110" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P110" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_geomorfologia_050203</v>
+      </c>
+      <c r="Q110" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_geomorfologia_050203.zip</v>
+      </c>
+    </row>
+    <row r="111" spans="1:17">
       <c r="A111">
         <v>143</v>
       </c>
@@ -6177,8 +7051,16 @@
       <c r="O111" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P111" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_geomorfologia_CA030</v>
+      </c>
+      <c r="Q111" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_geomorfologia_CA030.zip</v>
+      </c>
+    </row>
+    <row r="112" spans="1:17">
       <c r="A112">
         <v>144</v>
       </c>
@@ -6212,8 +7094,16 @@
       <c r="O112" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P112" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_DB200</v>
+      </c>
+      <c r="Q112" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_DB200.zip</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17">
       <c r="A113">
         <v>172</v>
       </c>
@@ -6247,8 +7137,16 @@
       <c r="O113" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P113" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_050204</v>
+      </c>
+      <c r="Q113" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_050204.zip</v>
+      </c>
+    </row>
+    <row r="114" spans="1:17">
       <c r="A114">
         <v>184</v>
       </c>
@@ -6282,8 +7180,16 @@
       <c r="O114" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P114" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_geomorfologia_CA025</v>
+      </c>
+      <c r="Q114" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_geomorfologia_CA025.zip</v>
+      </c>
+    </row>
+    <row r="115" spans="1:17">
       <c r="A115">
         <v>126</v>
       </c>
@@ -6317,8 +7223,16 @@
       <c r="O115" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P115" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_fabricacion_y_procesamiento_BH220</v>
+      </c>
+      <c r="Q115" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_fabricacion_y_procesamiento_BH220.zip</v>
+      </c>
+    </row>
+    <row r="116" spans="1:17">
       <c r="A116">
         <v>127</v>
       </c>
@@ -6352,8 +7266,16 @@
       <c r="O116" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P116" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_gestion_de_residuos_AB030</v>
+      </c>
+      <c r="Q116" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_gestion_de_residuos_AB030.zip</v>
+      </c>
+    </row>
+    <row r="117" spans="1:17">
       <c r="A117">
         <v>164</v>
       </c>
@@ -6387,8 +7309,16 @@
       <c r="O117" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P117" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_gestion_de_residuos_relleno_sanitario</v>
+      </c>
+      <c r="Q117" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_gestion_de_residuos_relleno_sanitario.zip</v>
+      </c>
+    </row>
+    <row r="118" spans="1:17">
       <c r="A118">
         <v>185</v>
       </c>
@@ -6422,8 +7352,16 @@
       <c r="O118" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P118" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_gestion_de_residuos_AB000</v>
+      </c>
+      <c r="Q118" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_gestion_de_residuos_AB000.zip</v>
+      </c>
+    </row>
+    <row r="119" spans="1:17">
       <c r="A119">
         <v>18</v>
       </c>
@@ -6457,8 +7395,16 @@
       <c r="O119" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P119" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_glaciologia_050705</v>
+      </c>
+      <c r="Q119" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_glaciologia_050705.zip</v>
+      </c>
+    </row>
+    <row r="120" spans="1:17">
       <c r="A120">
         <v>83</v>
       </c>
@@ -6492,8 +7438,16 @@
       <c r="O120" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P120" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_glaciologia_BJ030</v>
+      </c>
+      <c r="Q120" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_glaciologia_BJ030.zip</v>
+      </c>
+    </row>
+    <row r="121" spans="1:17">
       <c r="A121">
         <v>114</v>
       </c>
@@ -6527,8 +7481,16 @@
       <c r="O121" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P121" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_glaciologia_BJ020</v>
+      </c>
+      <c r="Q121" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_glaciologia_BJ020.zip</v>
+      </c>
+    </row>
+    <row r="122" spans="1:17">
       <c r="A122">
         <v>72</v>
       </c>
@@ -6562,8 +7524,16 @@
       <c r="O122" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P122" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>infraestructura_de_transporte_AQ125</v>
+      </c>
+      <c r="Q122" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/infraestructura_de_transporte_AQ125.zip</v>
+      </c>
+    </row>
+    <row r="123" spans="1:17">
       <c r="A123">
         <v>73</v>
       </c>
@@ -6597,8 +7567,16 @@
       <c r="O123" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P123" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>infraestructura_de_transporte_030801</v>
+      </c>
+      <c r="Q123" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/infraestructura_de_transporte_030801.zip</v>
+      </c>
+    </row>
+    <row r="124" spans="1:17">
       <c r="A124">
         <v>74</v>
       </c>
@@ -6632,8 +7610,16 @@
       <c r="O124" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P124" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>infraestructura_de_transporte_AQ180</v>
+      </c>
+      <c r="Q124" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/infraestructura_de_transporte_AQ180.zip</v>
+      </c>
+    </row>
+    <row r="125" spans="1:17">
       <c r="A125">
         <v>75</v>
       </c>
@@ -6667,8 +7653,16 @@
       <c r="O125" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P125" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>infraestructura_de_transporte_AQ170</v>
+      </c>
+      <c r="Q125" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/infraestructura_de_transporte_AQ170.zip</v>
+      </c>
+    </row>
+    <row r="126" spans="1:17">
       <c r="A126">
         <v>90</v>
       </c>
@@ -6702,8 +7696,16 @@
       <c r="O126" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P126" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>infraestructura_de_transporte_030803</v>
+      </c>
+      <c r="Q126" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/infraestructura_de_transporte_030803.zip</v>
+      </c>
+    </row>
+    <row r="127" spans="1:17">
       <c r="A127">
         <v>1</v>
       </c>
@@ -6737,8 +7739,16 @@
       <c r="O127" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P127" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>doscientas_millas_sector_antartico</v>
+      </c>
+      <c r="Q127" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/doscientas_millas_sector_antartico.zip</v>
+      </c>
+    </row>
+    <row r="128" spans="1:17">
       <c r="A128">
         <v>11</v>
       </c>
@@ -6772,8 +7782,16 @@
       <c r="O128" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P128" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>area_de_desarrollo_de_fronteras</v>
+      </c>
+      <c r="Q128" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/area_de_desarrollo_de_fronteras.zip</v>
+      </c>
+    </row>
+    <row r="129" spans="1:17">
       <c r="A129">
         <v>14</v>
       </c>
@@ -6807,8 +7825,16 @@
       <c r="O129" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P129" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>area_protegida</v>
+      </c>
+      <c r="Q129" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/area_protegida.zip</v>
+      </c>
+    </row>
+    <row r="130" spans="1:17">
       <c r="A130">
         <v>51</v>
       </c>
@@ -6842,8 +7868,16 @@
       <c r="O130" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P130" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>departamento</v>
+      </c>
+      <c r="Q130" s="5" t="str">
+        <f t="shared" ref="Q130:Q191" si="2">"https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/" &amp; P130 &amp; ".zip"</f>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/departamento.zip</v>
+      </c>
+    </row>
+    <row r="131" spans="1:17">
       <c r="A131">
         <v>84</v>
       </c>
@@ -6877,8 +7911,16 @@
       <c r="O131" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P131" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>gobiernoslocales_2022</v>
+      </c>
+      <c r="Q131" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/gobiernoslocales_2022.zip</v>
+      </c>
+    </row>
+    <row r="132" spans="1:17">
       <c r="A132">
         <v>85</v>
       </c>
@@ -6912,8 +7954,16 @@
       <c r="O132" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P132" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>municipio</v>
+      </c>
+      <c r="Q132" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/municipio.zip</v>
+      </c>
+    </row>
+    <row r="133" spans="1:17">
       <c r="A133">
         <v>87</v>
       </c>
@@ -6947,8 +7997,16 @@
       <c r="O133" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P133" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>hitos_internacionales</v>
+      </c>
+      <c r="Q133" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/hitos_internacionales.zip</v>
+      </c>
+    </row>
+    <row r="134" spans="1:17">
       <c r="A134">
         <v>88</v>
       </c>
@@ -6982,8 +8040,16 @@
       <c r="O134" t="s">
         <v>423</v>
       </c>
-    </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P134" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>hitos_interprovinciales</v>
+      </c>
+      <c r="Q134" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/hitos_interprovinciales.zip</v>
+      </c>
+    </row>
+    <row r="135" spans="1:17">
       <c r="A135">
         <v>96</v>
       </c>
@@ -7017,8 +8083,16 @@
       <c r="O135" t="s">
         <v>426</v>
       </c>
-    </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P135" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>linea_de_limite_070114</v>
+      </c>
+      <c r="Q135" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/linea_de_limite_070114.zip</v>
+      </c>
+    </row>
+    <row r="136" spans="1:17">
       <c r="A136">
         <v>97</v>
       </c>
@@ -7052,8 +8126,16 @@
       <c r="O136" t="s">
         <v>429</v>
       </c>
-    </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P136" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>linea_de_limite_070112</v>
+      </c>
+      <c r="Q136" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/linea_de_limite_070112.zip</v>
+      </c>
+    </row>
+    <row r="137" spans="1:17">
       <c r="A137">
         <v>98</v>
       </c>
@@ -7087,8 +8169,16 @@
       <c r="O137" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P137" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>linea_de_limite_070110</v>
+      </c>
+      <c r="Q137" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/linea_de_limite_070110.zip</v>
+      </c>
+    </row>
+    <row r="138" spans="1:17">
       <c r="A138">
         <v>99</v>
       </c>
@@ -7122,8 +8212,16 @@
       <c r="O138" t="s">
         <v>435</v>
       </c>
-    </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P138" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>linea_de_limite_FA004</v>
+      </c>
+      <c r="Q138" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/linea_de_limite_FA004.zip</v>
+      </c>
+    </row>
+    <row r="139" spans="1:17">
       <c r="A139">
         <v>100</v>
       </c>
@@ -7157,8 +8255,16 @@
       <c r="O139" t="s">
         <v>438</v>
       </c>
-    </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P139" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>linea_de_limite_070111</v>
+      </c>
+      <c r="Q139" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/linea_de_limite_070111.zip</v>
+      </c>
+    </row>
+    <row r="140" spans="1:17">
       <c r="A140">
         <v>101</v>
       </c>
@@ -7192,8 +8298,16 @@
       <c r="O140" t="s">
         <v>441</v>
       </c>
-    </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P140" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>linea_limite_maritimos</v>
+      </c>
+      <c r="Q140" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/linea_limite_maritimos.zip</v>
+      </c>
+    </row>
+    <row r="141" spans="1:17">
       <c r="A141">
         <v>105</v>
       </c>
@@ -7227,8 +8341,16 @@
       <c r="O141" t="s">
         <v>444</v>
       </c>
-    </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P141" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>mar_territorial_argentino</v>
+      </c>
+      <c r="Q141" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/mar_territorial_argentino.zip</v>
+      </c>
+    </row>
+    <row r="142" spans="1:17">
       <c r="A142">
         <v>117</v>
       </c>
@@ -7262,8 +8384,16 @@
       <c r="O142" t="s">
         <v>447</v>
       </c>
-    </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P142" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>pais</v>
+      </c>
+      <c r="Q142" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/pais.zip</v>
+      </c>
+    </row>
+    <row r="143" spans="1:17">
       <c r="A143">
         <v>133</v>
       </c>
@@ -7297,8 +8427,16 @@
       <c r="O143" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P143" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>plataforma_continental</v>
+      </c>
+      <c r="Q143" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/plataforma_continental.zip</v>
+      </c>
+    </row>
+    <row r="144" spans="1:17">
       <c r="A144">
         <v>138</v>
       </c>
@@ -7332,8 +8470,16 @@
       <c r="O144" t="s">
         <v>453</v>
       </c>
-    </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P144" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>provincia</v>
+      </c>
+      <c r="Q144" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/provincia.zip</v>
+      </c>
+    </row>
+    <row r="145" spans="1:17">
       <c r="A145">
         <v>187</v>
       </c>
@@ -7367,8 +8513,16 @@
       <c r="O145" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P145" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>zona_contigua_argentina</v>
+      </c>
+      <c r="Q145" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/zona_contigua_argentina.zip</v>
+      </c>
+    </row>
+    <row r="146" spans="1:17">
       <c r="A146">
         <v>189</v>
       </c>
@@ -7402,8 +8556,16 @@
       <c r="O146" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P146" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>zona_contigua_argentina</v>
+      </c>
+      <c r="Q146" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/zona_contigua_argentina.zip</v>
+      </c>
+    </row>
+    <row r="147" spans="1:17">
       <c r="A147">
         <v>190</v>
       </c>
@@ -7437,8 +8599,16 @@
       <c r="O147" t="s">
         <v>460</v>
       </c>
-    </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P147" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>zona_economica_exclusiva_argentina</v>
+      </c>
+      <c r="Q147" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/zona_economica_exclusiva_argentina.zip</v>
+      </c>
+    </row>
+    <row r="148" spans="1:17">
       <c r="A148">
         <v>106</v>
       </c>
@@ -7472,8 +8642,16 @@
       <c r="O148" t="s">
         <v>464</v>
       </c>
-    </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P148" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>mareas_y_corrientes_BG020</v>
+      </c>
+      <c r="Q148" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/mareas_y_corrientes_BG020.zip</v>
+      </c>
+    </row>
+    <row r="149" spans="1:17">
       <c r="A149">
         <v>165</v>
       </c>
@@ -7507,8 +8685,16 @@
       <c r="O149" t="s">
         <v>468</v>
       </c>
-    </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P149" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_obstrucciones_BD130</v>
+      </c>
+      <c r="Q149" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_obstrucciones_BD130.zip</v>
+      </c>
+    </row>
+    <row r="150" spans="1:17">
       <c r="A150">
         <v>115</v>
       </c>
@@ -7542,8 +8728,16 @@
       <c r="O150" t="s">
         <v>472</v>
       </c>
-    </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P150" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_puertos_y_muelles_BB190</v>
+      </c>
+      <c r="Q150" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_puertos_y_muelles_BB190.zip</v>
+      </c>
+    </row>
+    <row r="151" spans="1:17">
       <c r="A151">
         <v>141</v>
       </c>
@@ -7577,8 +8771,16 @@
       <c r="O151" t="s">
         <v>475</v>
       </c>
-    </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P151" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_puertos_y_muelles_BB005</v>
+      </c>
+      <c r="Q151" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_puertos_y_muelles_BB005.zip</v>
+      </c>
+    </row>
+    <row r="152" spans="1:17">
       <c r="A152">
         <v>166</v>
       </c>
@@ -7612,8 +8814,16 @@
       <c r="O152" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P152" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_puertos_y_muelles_BB041</v>
+      </c>
+      <c r="Q152" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_puertos_y_muelles_BB041.zip</v>
+      </c>
+    </row>
+    <row r="153" spans="1:17">
       <c r="A153">
         <v>167</v>
       </c>
@@ -7647,8 +8857,16 @@
       <c r="O153" t="s">
         <v>480</v>
       </c>
-    </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P153" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_puertos_y_muelles_BB041</v>
+      </c>
+      <c r="Q153" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_puertos_y_muelles_BB041.zip</v>
+      </c>
+    </row>
+    <row r="154" spans="1:17">
       <c r="A154">
         <v>39</v>
       </c>
@@ -7682,8 +8900,16 @@
       <c r="O154" t="s">
         <v>484</v>
       </c>
-    </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P154" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_terrestres_070401</v>
+      </c>
+      <c r="Q154" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_terrestres_070401.zip</v>
+      </c>
+    </row>
+    <row r="155" spans="1:17">
       <c r="A155">
         <v>55</v>
       </c>
@@ -7717,8 +8943,16 @@
       <c r="O155" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P155" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_terrestres_070403</v>
+      </c>
+      <c r="Q155" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_terrestres_070403.zip</v>
+      </c>
+    </row>
+    <row r="156" spans="1:17">
       <c r="A156">
         <v>180</v>
       </c>
@@ -7752,8 +8986,16 @@
       <c r="O156" t="s">
         <v>490</v>
       </c>
-    </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P156" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_terrestres_070402</v>
+      </c>
+      <c r="Q156" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_terrestres_070402.zip</v>
+      </c>
+    </row>
+    <row r="157" spans="1:17">
       <c r="A157">
         <v>37</v>
       </c>
@@ -7787,8 +9029,16 @@
       <c r="O157" t="s">
         <v>494</v>
       </c>
-    </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P157" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_recreacion_020401</v>
+      </c>
+      <c r="Q157" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_recreacion_020401.zip</v>
+      </c>
+    </row>
+    <row r="158" spans="1:17">
       <c r="A158">
         <v>91</v>
       </c>
@@ -7822,8 +9072,16 @@
       <c r="O158" t="s">
         <v>497</v>
       </c>
-    </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P158" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>puntos_de_recreacion_AK040</v>
+      </c>
+      <c r="Q158" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/puntos_de_recreacion_AK040.zip</v>
+      </c>
+    </row>
+    <row r="159" spans="1:17">
       <c r="A159">
         <v>145</v>
       </c>
@@ -7857,8 +9115,16 @@
       <c r="O159" t="s">
         <v>501</v>
       </c>
-    </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P159" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>ramsac</v>
+      </c>
+      <c r="Q159" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/ramsac.zip</v>
+      </c>
+    </row>
+    <row r="160" spans="1:17">
       <c r="A160">
         <v>146</v>
       </c>
@@ -7892,8 +9158,16 @@
       <c r="O160" t="s">
         <v>504</v>
       </c>
-    </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P160" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>nivelacion_alta_precision</v>
+      </c>
+      <c r="Q160" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/nivelacion_alta_precision.zip</v>
+      </c>
+    </row>
+    <row r="161" spans="1:17">
       <c r="A161">
         <v>147</v>
       </c>
@@ -7927,8 +9201,16 @@
       <c r="O161" t="s">
         <v>507</v>
       </c>
-    </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P161" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>nivelacion_precision</v>
+      </c>
+      <c r="Q161" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/nivelacion_precision.zip</v>
+      </c>
+    </row>
+    <row r="162" spans="1:17">
       <c r="A162">
         <v>148</v>
       </c>
@@ -7962,8 +9244,16 @@
       <c r="O162" t="s">
         <v>510</v>
       </c>
-    </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P162" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>nivelacion_topografica</v>
+      </c>
+      <c r="Q162" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/nivelacion_topografica.zip</v>
+      </c>
+    </row>
+    <row r="163" spans="1:17">
       <c r="A163">
         <v>149</v>
       </c>
@@ -7997,8 +9287,16 @@
       <c r="O163" t="s">
         <v>510</v>
       </c>
-    </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P163" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>nivelacion_topografica</v>
+      </c>
+      <c r="Q163" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/nivelacion_topografica.zip</v>
+      </c>
+    </row>
+    <row r="164" spans="1:17">
       <c r="A164">
         <v>150</v>
       </c>
@@ -8032,8 +9330,16 @@
       <c r="O164" t="s">
         <v>514</v>
       </c>
-    </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P164" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>red_pasma</v>
+      </c>
+      <c r="Q164" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/red_pasma.zip</v>
+      </c>
+    </row>
+    <row r="165" spans="1:17">
       <c r="A165">
         <v>151</v>
       </c>
@@ -8067,8 +9373,16 @@
       <c r="O165" t="s">
         <v>517</v>
       </c>
-    </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P165" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>red_posgar</v>
+      </c>
+      <c r="Q165" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/red_posgar.zip</v>
+      </c>
+    </row>
+    <row r="166" spans="1:17">
       <c r="A166">
         <v>152</v>
       </c>
@@ -8102,8 +9416,16 @@
       <c r="O166" t="s">
         <v>520</v>
       </c>
-    </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P166" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>red_provincial</v>
+      </c>
+      <c r="Q166" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/red_provincial.zip</v>
+      </c>
+    </row>
+    <row r="167" spans="1:17">
       <c r="A167">
         <v>153</v>
       </c>
@@ -8137,8 +9459,16 @@
       <c r="O167" t="s">
         <v>523</v>
       </c>
-    </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P167" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>gravimetria_bacara</v>
+      </c>
+      <c r="Q167" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/gravimetria_bacara.zip</v>
+      </c>
+    </row>
+    <row r="168" spans="1:17">
       <c r="A168">
         <v>154</v>
       </c>
@@ -8172,8 +9502,16 @@
       <c r="O168" t="s">
         <v>526</v>
       </c>
-    </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P168" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>gravimetria_rpo</v>
+      </c>
+      <c r="Q168" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/gravimetria_rpo.zip</v>
+      </c>
+    </row>
+    <row r="169" spans="1:17">
       <c r="A169">
         <v>155</v>
       </c>
@@ -8204,11 +9542,19 @@
       <c r="N169" t="s">
         <v>528</v>
       </c>
-      <c r="O169" t="s">
+      <c r="O169" s="4" t="s">
         <v>529</v>
       </c>
-    </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P169" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>gravimetria_rso</v>
+      </c>
+      <c r="Q169" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/gravimetria_rso.zip</v>
+      </c>
+    </row>
+    <row r="170" spans="1:17">
       <c r="A170">
         <v>156</v>
       </c>
@@ -8242,8 +9588,16 @@
       <c r="O170" t="s">
         <v>532</v>
       </c>
-    </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P170" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>gravimetria_rto</v>
+      </c>
+      <c r="Q170" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/gravimetria_rto.zip</v>
+      </c>
+    </row>
+    <row r="171" spans="1:17">
       <c r="A171">
         <v>157</v>
       </c>
@@ -8277,8 +9631,16 @@
       <c r="O171" t="s">
         <v>535</v>
       </c>
-    </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P171" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>gravimetria_igsn71</v>
+      </c>
+      <c r="Q171" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/gravimetria_igsn71.zip</v>
+      </c>
+    </row>
+    <row r="172" spans="1:17">
       <c r="A172">
         <v>158</v>
       </c>
@@ -8312,8 +9674,16 @@
       <c r="O172" t="s">
         <v>538</v>
       </c>
-    </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P172" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>gravimetria_raga</v>
+      </c>
+      <c r="Q172" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/gravimetria_raga.zip</v>
+      </c>
+    </row>
+    <row r="173" spans="1:17">
       <c r="A173">
         <v>159</v>
       </c>
@@ -8344,11 +9714,19 @@
       <c r="N173" t="s">
         <v>540</v>
       </c>
-      <c r="O173" t="s">
+      <c r="O173" s="4" t="s">
         <v>541</v>
       </c>
-    </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P173" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>ramsac_ntrip</v>
+      </c>
+      <c r="Q173" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/ramsac_ntrip.zip</v>
+      </c>
+    </row>
+    <row r="174" spans="1:17">
       <c r="A174">
         <v>59</v>
       </c>
@@ -8382,8 +9760,16 @@
       <c r="O174" t="s">
         <v>545</v>
       </c>
-    </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P174" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>salud_020801</v>
+      </c>
+      <c r="Q174" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/salud_020801.zip</v>
+      </c>
+    </row>
+    <row r="175" spans="1:17">
       <c r="A175">
         <v>52</v>
       </c>
@@ -8405,8 +9791,16 @@
       <c r="O175" t="s">
         <v>549</v>
       </c>
-    </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P175" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>sin_vegetacion_061001</v>
+      </c>
+      <c r="Q175" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/sin_vegetacion_061001.zip</v>
+      </c>
+    </row>
+    <row r="176" spans="1:17">
       <c r="A176">
         <v>21</v>
       </c>
@@ -8428,8 +9822,16 @@
       <c r="O176" t="s">
         <v>553</v>
       </c>
-    </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P176" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vegetacion_arborea_060301</v>
+      </c>
+      <c r="Q176" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vegetacion_arborea_060301.zip</v>
+      </c>
+    </row>
+    <row r="177" spans="1:17">
       <c r="A177">
         <v>22</v>
       </c>
@@ -8451,8 +9853,16 @@
       <c r="O177" t="s">
         <v>556</v>
       </c>
-    </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P177" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vegetacion_arborea_EC015</v>
+      </c>
+      <c r="Q177" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vegetacion_arborea_EC015.zip</v>
+      </c>
+    </row>
+    <row r="178" spans="1:17">
       <c r="A178">
         <v>112</v>
       </c>
@@ -8474,8 +9884,16 @@
       <c r="O178" t="s">
         <v>559</v>
       </c>
-    </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P178" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vegetacion_arborea_060302</v>
+      </c>
+      <c r="Q178" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vegetacion_arborea_060302.zip</v>
+      </c>
+    </row>
+    <row r="179" spans="1:17">
       <c r="A179">
         <v>120</v>
       </c>
@@ -8497,8 +9915,16 @@
       <c r="O179" t="s">
         <v>562</v>
       </c>
-    </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P179" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vegetacion_arborea_AK120</v>
+      </c>
+      <c r="Q179" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vegetacion_arborea_AK120.zip</v>
+      </c>
+    </row>
+    <row r="180" spans="1:17">
       <c r="A180">
         <v>76</v>
       </c>
@@ -8520,8 +9946,16 @@
       <c r="O180" t="s">
         <v>566</v>
       </c>
-    </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P180" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vegetacion_arbustiva_EB015</v>
+      </c>
+      <c r="Q180" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vegetacion_arbustiva_EB015.zip</v>
+      </c>
+    </row>
+    <row r="181" spans="1:17">
       <c r="A181">
         <v>118</v>
       </c>
@@ -8543,8 +9977,16 @@
       <c r="O181" t="s">
         <v>570</v>
       </c>
-    </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P181" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vegetacion_hidrofila_ED020</v>
+      </c>
+      <c r="Q181" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vegetacion_hidrofila_ED020.zip</v>
+      </c>
+    </row>
+    <row r="182" spans="1:17">
       <c r="A182">
         <v>89</v>
       </c>
@@ -8578,8 +10020,16 @@
       <c r="O182" t="s">
         <v>574</v>
       </c>
-    </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P182" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vial_AP010</v>
+      </c>
+      <c r="Q182" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vial_AP010.zip</v>
+      </c>
+    </row>
+    <row r="183" spans="1:17">
       <c r="A183">
         <v>160</v>
       </c>
@@ -8613,8 +10063,16 @@
       <c r="O183" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P183" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vial_nacional</v>
+      </c>
+      <c r="Q183" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vial_nacional.zip</v>
+      </c>
+    </row>
+    <row r="184" spans="1:17">
       <c r="A184">
         <v>161</v>
       </c>
@@ -8648,8 +10106,16 @@
       <c r="O184" t="s">
         <v>580</v>
       </c>
-    </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P184" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vial_provincial</v>
+      </c>
+      <c r="Q184" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vial_provincial.zip</v>
+      </c>
+    </row>
+    <row r="185" spans="1:17">
       <c r="A185">
         <v>162</v>
       </c>
@@ -8683,8 +10149,16 @@
       <c r="O185" t="s">
         <v>583</v>
       </c>
-    </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P185" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vial_terciaria</v>
+      </c>
+      <c r="Q185" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vial_terciaria.zip</v>
+      </c>
+    </row>
+    <row r="186" spans="1:17">
       <c r="A186">
         <v>171</v>
       </c>
@@ -8718,8 +10192,16 @@
       <c r="O186" t="s">
         <v>583</v>
       </c>
-    </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P186" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>vial_terciaria</v>
+      </c>
+      <c r="Q186" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/vial_terciaria.zip</v>
+      </c>
+    </row>
+    <row r="187" spans="1:17">
       <c r="A187">
         <v>3</v>
       </c>
@@ -8753,8 +10235,16 @@
       <c r="O187" t="s">
         <v>588</v>
       </c>
-    </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P187" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>lineas_de_zona_costera_BA040</v>
+      </c>
+      <c r="Q187" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/lineas_de_zona_costera_BA040.zip</v>
+      </c>
+    </row>
+    <row r="188" spans="1:17">
       <c r="A188">
         <v>95</v>
       </c>
@@ -8788,8 +10278,16 @@
       <c r="O188" t="s">
         <v>591</v>
       </c>
-    </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P188" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_zona_costera_BA030</v>
+      </c>
+      <c r="Q188" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_zona_costera_BA030.zip</v>
+      </c>
+    </row>
+    <row r="189" spans="1:17">
       <c r="A189">
         <v>134</v>
       </c>
@@ -8823,8 +10321,16 @@
       <c r="O189" t="s">
         <v>594</v>
       </c>
-    </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P189" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_zona_costera_playa_areana</v>
+      </c>
+      <c r="Q189" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_zona_costera_playa_areana.zip</v>
+      </c>
+    </row>
+    <row r="190" spans="1:17">
       <c r="A190">
         <v>135</v>
       </c>
@@ -8858,8 +10364,16 @@
       <c r="O190" t="s">
         <v>597</v>
       </c>
-    </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P190" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_zona_costera_playa_grava</v>
+      </c>
+      <c r="Q190" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_zona_costera_playa_grava.zip</v>
+      </c>
+    </row>
+    <row r="191" spans="1:17">
       <c r="A191">
         <v>136</v>
       </c>
@@ -8892,6 +10406,14 @@
       </c>
       <c r="O191" t="s">
         <v>600</v>
+      </c>
+      <c r="P191" t="str">
+        <f>MID(Tabla1[[#This Row],[Link CSV]],102,LEN(Tabla1[[#This Row],[Link CSV]])-118)</f>
+        <v>areas_de_zona_costera_playa_restinga</v>
+      </c>
+      <c r="Q191" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>https://github.com/Luthcibel/Carto_a_la_Carta/raw/refs/heads/main/datos_csv/areas_de_zona_costera_playa_restinga.zip</v>
       </c>
     </row>
   </sheetData>
@@ -8903,9 +10425,14 @@
       <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="O2" r:id="rId1"/>
+    <hyperlink ref="O173" r:id="rId2"/>
+    <hyperlink ref="O169" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>